<commit_message>
docs: update test plan for v1.0.0 with X-Checks strategy
- 5 new X-Checks workflow cases
- Files Required rows for X-Checks (4 fields incl. 2 optional)
- Dropdown count updated to 5
- Full Run sheet counts and strategy order updated
- Upload dialog titles updated

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/20260630 X-Checks_v1.0.0 Test Plan.xlsx
+++ b/docs/20260630 X-Checks_v1.0.0 Test Plan.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45.7" customWidth="1" min="1" max="1"/>
@@ -497,138 +497,133 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Task selector launcher — dropdown lists all four strategies; Start button disabled until selection made.</t>
+          <t>Task selector launcher — dropdown lists all five strategies; Start button disabled until selection made.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>File upload dialog — dynamically built from config; sheet name fields enabled on file select.</t>
+          <t>X-Checks strategy — compares EBX cross-check formulas and variables against FIP validation rules; flags differences and known exceptions.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Sheet name advisory label — displayed when any field has a sheet name input.</t>
+          <t>File upload dialog — dynamically built from config; sheet name fields enabled on file select.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Grouping By strategy — compares X-Check grouping data (EBX publication) against FIP ZQ9_VALFLDGR extract.</t>
+          <t>Sheet name advisory label — displayed when any field has a sheet name input.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Accounting Principles strategy — compares severity letters (W/E) from EBX publication against FIP VALMSG.</t>
+          <t>Grouping By strategy — compares X-Check grouping data (EBX publication) against FIP ZQ9_VALFLDGR extract.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Conditions strategy — matches X-Check|Condition pairs from EBX publication against FIP ZQ9_VALMETH.</t>
+          <t>Accounting Principles strategy — compares severity letters (W/E) from EBX publication against FIP VALMSG.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Full Run strategy — runs all three strategies sequentially and combines output into one colour-coded workbook.</t>
+          <t>Conditions strategy — matches X-Check|Condition pairs from EBX publication against FIP ZQ9_VALMETH.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Progress dialog — real-time scrollable log; error lines in bold red; Stop / Return to Form / Exit buttons.</t>
+          <t>Full Run strategy — runs all three strategies sequentially and combines output into one colour-coded workbook.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sensitivity labelling — Microsoft Information Protection label applied automatically to every output workbook.</t>
+          <t>Progress dialog — real-time scrollable log; error lines in bold red; Stop / Return to Form / Exit buttons.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>Sensitivity labelling — Microsoft Information Protection label applied automatically to every output workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
           <t>Output to ~/Downloads/Output — all runs write to the same folder for easy access.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Test Plan</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>Test Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Expected result</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Tested Date</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>App launches</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Double-click X-Checks_v1.0.0.exe.</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Splash screen appears showing version v1.0.0.</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Splash closes and the task selector dialog opens showing 'X-Check Application v1.0.0'.</t>
         </is>
       </c>
       <c r="D16" s="4" t="n"/>
@@ -640,7 +635,7 @@
       <c r="B17" s="4" t="n"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Dropdown lists exactly four options: Grouping By, Accounting Principles, Conditions, Full Run.</t>
+          <t>Splash closes and the task selector dialog opens showing 'X-Check Application v1.0.0'.</t>
         </is>
       </c>
       <c r="D17" s="4" t="n"/>
@@ -652,7 +647,7 @@
       <c r="B18" s="4" t="n"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Start button is disabled until an option is selected.</t>
+          <t>Dropdown lists exactly five options: X-Checks, Grouping By, Accounting Principles, Conditions, Full Run.</t>
         </is>
       </c>
       <c r="D18" s="4" t="n"/>
@@ -660,19 +655,11 @@
       <c r="F18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Task selector — select task</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Select any task from the dropdown.</t>
-        </is>
-      </c>
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="n"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Start button becomes enabled.</t>
+          <t>Start button is disabled until an option is selected.</t>
         </is>
       </c>
       <c r="D19" s="4" t="n"/>
@@ -682,17 +669,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Task selector — close</t>
+          <t>Task selector — select task</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Click the red X on the task selector.</t>
+          <t>Select any task from the dropdown.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Application closes cleanly with no error.</t>
+          <t>Start button becomes enabled.</t>
         </is>
       </c>
       <c r="D20" s="4" t="n"/>
@@ -702,17 +689,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>File upload dialog opens</t>
+          <t>Task selector — close</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Select 'Grouping By' and click Start.</t>
+          <t>Click the red X on the task selector.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>File upload dialog opens titled 'Grouping By Files'.</t>
+          <t>Application closes cleanly with no error.</t>
         </is>
       </c>
       <c r="D21" s="4" t="n"/>
@@ -720,11 +707,19 @@
       <c r="F21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>File upload dialog opens</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Select 'Grouping By' and click Start.</t>
+        </is>
+      </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Required field labels show a trailing asterisk (*); optional fields show '(optional)'.</t>
+          <t>File upload dialog opens titled 'Grouping By Files'.</t>
         </is>
       </c>
       <c r="D22" s="4" t="n"/>
@@ -736,7 +731,7 @@
       <c r="B23" s="4" t="n"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>All file path labels show 'No file selected' in grey.</t>
+          <t>Required field labels show a trailing asterisk (*); optional fields show '(optional)'.</t>
         </is>
       </c>
       <c r="D23" s="4" t="n"/>
@@ -748,7 +743,7 @@
       <c r="B24" s="4" t="n"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Sheet name fields are greyed out / disabled.</t>
+          <t>All file path labels show 'No file selected' in grey.</t>
         </is>
       </c>
       <c r="D24" s="4" t="n"/>
@@ -760,7 +755,7 @@
       <c r="B25" s="4" t="n"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Advisory note 'If the sheet name changes from the current default in the Excel workbook, update it manually.' is visible, centred.</t>
+          <t>Sheet name fields are greyed out / disabled.</t>
         </is>
       </c>
       <c r="D25" s="4" t="n"/>
@@ -772,7 +767,7 @@
       <c r="B26" s="4" t="n"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Proceed button is disabled.</t>
+          <t>Advisory note 'If the sheet name changes from the current default in the Excel workbook, update it manually.' is visible, centred.</t>
         </is>
       </c>
       <c r="D26" s="4" t="n"/>
@@ -780,19 +775,11 @@
       <c r="F26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Browse — file select</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Click Browse next to 'FIP File (ZQ9_VALFLDGR)' and select the VALFLDGR test file.</t>
-        </is>
-      </c>
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="4" t="n"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>File path label updates to the filename (not full path).</t>
+          <t>Proceed button is disabled.</t>
         </is>
       </c>
       <c r="D27" s="4" t="n"/>
@@ -800,11 +787,19 @@
       <c r="F27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="n"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Browse — file select</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Click Browse next to 'FIP File (ZQ9_VALFLDGR)' and select the VALFLDGR test file.</t>
+        </is>
+      </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Sheet name field for that row becomes enabled.</t>
+          <t>File path label updates to the filename (not full path).</t>
         </is>
       </c>
       <c r="D28" s="4" t="n"/>
@@ -816,7 +811,7 @@
       <c r="B29" s="4" t="n"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Proceed button remains disabled (other required files not yet provided).</t>
+          <t>Sheet name field for that row becomes enabled.</t>
         </is>
       </c>
       <c r="D29" s="4" t="n"/>
@@ -824,19 +819,11 @@
       <c r="F29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Proceed enables</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Select valid files for all required fields and an output directory.</t>
-        </is>
-      </c>
+      <c r="A30" s="4" t="n"/>
+      <c r="B30" s="4" t="n"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Proceed button becomes enabled.</t>
+          <t>Proceed button remains disabled (other required files not yet provided).</t>
         </is>
       </c>
       <c r="D30" s="4" t="n"/>
@@ -846,17 +833,17 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Cancel dialog</t>
+          <t>Proceed enables</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Close the upload dialog using the red X.</t>
+          <t>Select valid files for all required fields and an output directory.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Task selector reappears.</t>
+          <t>Proceed button becomes enabled.</t>
         </is>
       </c>
       <c r="D31" s="4" t="n"/>
@@ -866,17 +853,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Grouping By — run (debug EXE)</t>
+          <t>Cancel dialog</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Run X-Checks_Debug_GroupingBy_v1.0.0.exe.</t>
+          <t>Close the upload dialog using the red X.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>App launches in debug mode; progress dialog opens immediately with pre-loaded test files.</t>
+          <t>Task selector reappears.</t>
         </is>
       </c>
       <c r="D32" s="4" t="n"/>
@@ -884,11 +871,19 @@
       <c r="F32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n"/>
-      <c r="B33" s="4" t="n"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>X-Checks — run (debug EXE)</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Run X-Checks_Debug_XChecks_v1.0.0.exe.</t>
+        </is>
+      </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Progress log shows 'Loading files into memory...' then 'Files loaded successfully'.</t>
+          <t>App launches in debug mode; progress dialog opens immediately with pre-loaded test files.</t>
         </is>
       </c>
       <c r="D33" s="4" t="n"/>
@@ -900,7 +895,7 @@
       <c r="B34" s="4" t="n"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Log shows EBX processing steps: Original file loaded → Filtered → Deduplicated → Split → Stacked.</t>
+          <t>Progress log shows 'Loading files into memory...' then 'Files loaded successfully'.</t>
         </is>
       </c>
       <c r="D34" s="4" t="n"/>
@@ -912,7 +907,7 @@
       <c r="B35" s="4" t="n"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Log shows Compare result: 'Matched: N | Not in FIP: M' with N &gt; 0.</t>
+          <t>Log shows EBX extraction steps, FIP extraction steps, then comparison.</t>
         </is>
       </c>
       <c r="D35" s="4" t="n"/>
@@ -948,7 +943,7 @@
       <c r="B38" s="4" t="n"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Workbook contains 7 sheets: Mapping File, FIP - Original, FIP - Processed, EBX - Original, EBX - Processed, Compare, Processing Log.</t>
+          <t>Workbook contains 2 sheets: X-Checks Comparison, Processing Log.</t>
         </is>
       </c>
       <c r="D38" s="4" t="n"/>
@@ -960,7 +955,7 @@
       <c r="B39" s="4" t="n"/>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Compare sheet has a 'Result' column with values 'Matched' and/or 'Not in FIP'.</t>
+          <t>X-Checks Comparison sheet has a 'Result' column with colour-coded values (Matched / MisMatch / Not Found etc.).</t>
         </is>
       </c>
       <c r="D39" s="4" t="n"/>
@@ -970,17 +965,17 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Accounting Principles — run (debug EXE)</t>
+          <t>Grouping By — run (debug EXE)</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Run X-Checks_Debug_AccountingPrinciples_v1.0.0.exe.</t>
+          <t>Run X-Checks_Debug_GroupingBy_v1.0.0.exe.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>App launches in debug mode; progress dialog opens with pre-loaded test files.</t>
+          <t>App launches in debug mode; progress dialog opens immediately with pre-loaded test files.</t>
         </is>
       </c>
       <c r="D40" s="4" t="n"/>
@@ -992,7 +987,7 @@
       <c r="B41" s="4" t="n"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Log shows 'Validation Methods — Method bindings extracted N' with N &gt; 0.</t>
+          <t>Progress log shows 'Loading files into memory...' then 'Files loaded successfully'.</t>
         </is>
       </c>
       <c r="D41" s="4" t="n"/>
@@ -1004,7 +999,7 @@
       <c r="B42" s="4" t="n"/>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Log shows 'EBX — In-scope X-Check Nos N'.</t>
+          <t>Log shows EBX processing steps: Original file loaded → Filtered → Deduplicated → Split → Stacked.</t>
         </is>
       </c>
       <c r="D42" s="4" t="n"/>
@@ -1016,7 +1011,7 @@
       <c r="B43" s="4" t="n"/>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Log shows 'Compare — Comparison rows produced N'.</t>
+          <t>Log shows Compare result: 'Matched: N | Not in FIP: M' with N &gt; 0.</t>
         </is>
       </c>
       <c r="D43" s="4" t="n"/>
@@ -1040,7 +1035,7 @@
       <c r="B45" s="4" t="n"/>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Output workbook written to ~/Downloads/Output/.</t>
+          <t>Output workbook written to ~/Downloads/Output/ with timestamp prefix.</t>
         </is>
       </c>
       <c r="D45" s="4" t="n"/>
@@ -1052,7 +1047,7 @@
       <c r="B46" s="4" t="n"/>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Workbook contains 4 sheets: EBX, FIP, Comparison, Processing Log.</t>
+          <t>Workbook contains 7 sheets: Mapping File, FIP - Original, FIP - Processed, EBX - Original, EBX - Processed, Compare, Processing Log.</t>
         </is>
       </c>
       <c r="D46" s="4" t="n"/>
@@ -1064,7 +1059,7 @@
       <c r="B47" s="4" t="n"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Comparison sheet has green rows (Match) and/or red rows (MisMatch).</t>
+          <t>Compare sheet has a 'Result' column with values 'Matched' and/or 'Not in FIP'.</t>
         </is>
       </c>
       <c r="D47" s="4" t="n"/>
@@ -1074,12 +1069,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Conditions — run (debug EXE)</t>
+          <t>Accounting Principles — run (debug EXE)</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Run X-Checks_Debug_Conditions_v1.0.0.exe.</t>
+          <t>Run X-Checks_Debug_AccountingPrinciples_v1.0.0.exe.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -1096,7 +1091,7 @@
       <c r="B49" s="4" t="n"/>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Log shows 'Publication — Extracted N unique X-Check No. entries'.</t>
+          <t>Log shows 'Validation Methods — Method bindings extracted N' with N &gt; 0.</t>
         </is>
       </c>
       <c r="D49" s="4" t="n"/>
@@ -1108,7 +1103,7 @@
       <c r="B50" s="4" t="n"/>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Log shows 'Comparison — Pairs checked: N, Matched: M, Not matched: P'.</t>
+          <t>Log shows 'EBX — In-scope X-Check Nos N'.</t>
         </is>
       </c>
       <c r="D50" s="4" t="n"/>
@@ -1120,7 +1115,7 @@
       <c r="B51" s="4" t="n"/>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Log ends with 'Processing complete. You may close this window.'</t>
+          <t>Log shows 'Compare — Comparison rows produced N'.</t>
         </is>
       </c>
       <c r="D51" s="4" t="n"/>
@@ -1132,7 +1127,7 @@
       <c r="B52" s="4" t="n"/>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Output workbook written to ~/Downloads/Output/.</t>
+          <t>Log ends with 'Processing complete. You may close this window.'</t>
         </is>
       </c>
       <c r="D52" s="4" t="n"/>
@@ -1144,7 +1139,7 @@
       <c r="B53" s="4" t="n"/>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Workbook contains 4 sheets: Conditions, Working Sheet, FIP Data, Processing Log.</t>
+          <t>Output workbook written to ~/Downloads/Output/.</t>
         </is>
       </c>
       <c r="D53" s="4" t="n"/>
@@ -1156,7 +1151,7 @@
       <c r="B54" s="4" t="n"/>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Conditions sheet has a summary block at the top and TRUE/FALSE rows below.</t>
+          <t>Workbook contains 4 sheets: EBX, FIP, Comparison, Processing Log.</t>
         </is>
       </c>
       <c r="D54" s="4" t="n"/>
@@ -1164,19 +1159,11 @@
       <c r="F54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Full Run — run (debug EXE)</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Run X-Checks_Debug_FullRun_v1.0.0.exe.</t>
-        </is>
-      </c>
+      <c r="A55" s="4" t="n"/>
+      <c r="B55" s="4" t="n"/>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>App launches in debug mode; progress dialog opens with pre-loaded test files.</t>
+          <t>Comparison sheet has green rows (Match) and/or red rows (MisMatch).</t>
         </is>
       </c>
       <c r="D55" s="4" t="n"/>
@@ -1184,11 +1171,19 @@
       <c r="F55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="n"/>
-      <c r="B56" s="4" t="n"/>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Conditions — run (debug EXE)</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Run X-Checks_Debug_Conditions_v1.0.0.exe.</t>
+        </is>
+      </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Log shows '— Starting: Grouping By —', then '— Starting: Accounting Principles —', then '— Starting: Conditions —' in order.</t>
+          <t>App launches in debug mode; progress dialog opens with pre-loaded test files.</t>
         </is>
       </c>
       <c r="D56" s="4" t="n"/>
@@ -1200,7 +1195,7 @@
       <c r="B57" s="4" t="n"/>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Log shows 'Writing combined workbook (12 sheets)'.</t>
+          <t>Log shows 'Publication — Extracted N unique X-Check No. entries'.</t>
         </is>
       </c>
       <c r="D57" s="4" t="n"/>
@@ -1212,7 +1207,7 @@
       <c r="B58" s="4" t="n"/>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Log ends with 'Processing complete. You may close this window.'</t>
+          <t>Log shows 'Comparison — Pairs checked: N, Matched: M, Not matched: P'.</t>
         </is>
       </c>
       <c r="D58" s="4" t="n"/>
@@ -1224,7 +1219,7 @@
       <c r="B59" s="4" t="n"/>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Single output workbook written to ~/Downloads/Output/.</t>
+          <t>Log ends with 'Processing complete. You may close this window.'</t>
         </is>
       </c>
       <c r="D59" s="4" t="n"/>
@@ -1236,7 +1231,7 @@
       <c r="B60" s="4" t="n"/>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Workbook contains 13 sheets: 6 GB tabs (orange), 3 AP tabs (dark blue), 3 Cond tabs (blue), 1 Processing Log (grey).</t>
+          <t>Output workbook written to ~/Downloads/Output/.</t>
         </is>
       </c>
       <c r="D60" s="4" t="n"/>
@@ -1248,7 +1243,7 @@
       <c r="B61" s="4" t="n"/>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Tab colours match Zurich brand palette: Grouping By = orange, Accounting Principles = dark blue, Conditions = Zurich blue.</t>
+          <t>Workbook contains 4 sheets: Conditions, Working Sheet, FIP Data, Processing Log.</t>
         </is>
       </c>
       <c r="D61" s="4" t="n"/>
@@ -1256,19 +1251,11 @@
       <c r="F61" s="4" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Wrong sheet name</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>In the upload dialog, change a sheet name to a name that does not exist in the file, then click Proceed.</t>
-        </is>
-      </c>
+      <c r="A62" s="4" t="n"/>
+      <c r="B62" s="4" t="n"/>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Progress dialog opens and immediately shows an error: 'Could not find sheet … in …'.</t>
+          <t>Conditions sheet has a summary block at the top and TRUE/FALSE rows below.</t>
         </is>
       </c>
       <c r="D62" s="4" t="n"/>
@@ -1276,11 +1263,19 @@
       <c r="F62" s="4" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="4" t="n"/>
-      <c r="B63" s="4" t="n"/>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Full Run — run (debug EXE)</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Run X-Checks_Debug_FullRun_v1.0.0.exe.</t>
+        </is>
+      </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>'Return to Form' button appears; clicking it re-opens the upload dialog with previous inputs pre-filled.</t>
+          <t>App launches in debug mode; progress dialog opens with pre-loaded test files.</t>
         </is>
       </c>
       <c r="D63" s="4" t="n"/>
@@ -1288,19 +1283,11 @@
       <c r="F63" s="4" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Stop mid-run</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Start a run (e.g. Full Run) and click Stop during processing.</t>
-        </is>
-      </c>
+      <c r="A64" s="4" t="n"/>
+      <c r="B64" s="4" t="n"/>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Processing halts after the current step completes.</t>
+          <t>Log shows '— Starting: Grouping By —', then '— Starting: Accounting Principles —', then '— Starting: Conditions —' in order.</t>
         </is>
       </c>
       <c r="D64" s="4" t="n"/>
@@ -1312,7 +1299,7 @@
       <c r="B65" s="4" t="n"/>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Log shows 'Processing halted by user.'</t>
+          <t>Log shows 'Writing combined workbook (12 sheets)'.</t>
         </is>
       </c>
       <c r="D65" s="4" t="n"/>
@@ -1324,7 +1311,7 @@
       <c r="B66" s="4" t="n"/>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>'Return to Form' button appears.</t>
+          <t>Log ends with 'Processing complete. You may close this window.'</t>
         </is>
       </c>
       <c r="D66" s="4" t="n"/>
@@ -1332,19 +1319,11 @@
       <c r="F66" s="4" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>Version displayed</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Inspect the title bar of the task selector and the first line of any processing log.</t>
-        </is>
-      </c>
+      <c r="A67" s="4" t="n"/>
+      <c r="B67" s="4" t="n"/>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Title bar reads 'X-Check Application v1.0.0'.</t>
+          <t>Single output workbook written to ~/Downloads/Output/.</t>
         </is>
       </c>
       <c r="D67" s="4" t="n"/>
@@ -1356,12 +1335,132 @@
       <c r="B68" s="4" t="n"/>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>First log entry reads 'System — X-Check Application v1.0.0'.</t>
+          <t>Workbook contains 13 sheets: 6 GB tabs (orange), 3 AP tabs (dark blue), 3 Cond tabs (blue), 1 Processing Log (grey).</t>
         </is>
       </c>
       <c r="D68" s="4" t="n"/>
       <c r="E68" s="4" t="n"/>
       <c r="F68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="n"/>
+      <c r="B69" s="4" t="n"/>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Tab colours match Zurich brand palette: Grouping By = orange, Accounting Principles = dark blue, Conditions = Zurich blue.</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="n"/>
+      <c r="E69" s="4" t="n"/>
+      <c r="F69" s="4" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Wrong sheet name</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>In the upload dialog, change a sheet name to a name that does not exist in the file, then click Proceed.</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Progress dialog opens and immediately shows an error: 'Could not find sheet … in …'.</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="n"/>
+      <c r="E70" s="4" t="n"/>
+      <c r="F70" s="4" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="n"/>
+      <c r="B71" s="4" t="n"/>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>'Return to Form' button appears; clicking it re-opens the upload dialog with previous inputs pre-filled.</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="n"/>
+      <c r="E71" s="4" t="n"/>
+      <c r="F71" s="4" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Stop mid-run</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Start a run (e.g. Full Run) and click Stop during processing.</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Processing halts after the current step completes.</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="n"/>
+      <c r="E72" s="4" t="n"/>
+      <c r="F72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="n"/>
+      <c r="B73" s="4" t="n"/>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Log shows 'Processing halted by user.'</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="n"/>
+      <c r="E73" s="4" t="n"/>
+      <c r="F73" s="4" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n"/>
+      <c r="B74" s="4" t="n"/>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>'Return to Form' button appears.</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="n"/>
+      <c r="E74" s="4" t="n"/>
+      <c r="F74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Version displayed</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Inspect the title bar of the task selector and the first line of any processing log.</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Title bar reads 'X-Check Application v1.0.0'.</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="n"/>
+      <c r="E75" s="4" t="n"/>
+      <c r="F75" s="4" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n"/>
+      <c r="B76" s="4" t="n"/>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>First log entry reads 'System — X-Check Application v1.0.0'.</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="n"/>
+      <c r="E76" s="4" t="n"/>
+      <c r="F76" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1374,7 +1473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19.4" customWidth="1" min="1" max="1"/>
@@ -1424,22 +1523,22 @@
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Grouping By</t>
+          <t>X-Checks</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>FIP File (ZQ9_VALFLDGR)</t>
+          <t>FIP file</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>VALFLDGR file with 12348 Data rows on sheet Sheet1.XLSX</t>
+          <t>20260318 FIP X-Checks.txt</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Sheet1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -1451,7 +1550,7 @@
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Grouping By</t>
+          <t>X-Checks</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
@@ -1478,76 +1577,76 @@
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Grouping By</t>
+          <t>X-Checks</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Mapping File</t>
+          <t>GCoA Publication File</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Mapping Table with 20 rows.txt</t>
+          <t>GCoA Publication file (optional)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>GCoA Base account table</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Accounting Principles</t>
+          <t>X-Checks</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Validation Methods File</t>
+          <t>Known Exception List</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>validation methods.xlsx</t>
+          <t>Known Exception List (optional)</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Validation Methods</t>
+          <t>Known Exceptions</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Accounting Principles</t>
+          <t>Grouping By</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>X-Checks Publication File</t>
+          <t>FIP File (ZQ9_VALFLDGR)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>20260602 VALMSG (Accounting Principle).xlsx</t>
+          <t>VALFLDGR file with 12348 Data rows on sheet Sheet1.XLSX</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>cross checks all</t>
+          <t>Sheet1</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1559,22 +1658,22 @@
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Accounting Principles</t>
+          <t>Grouping By</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>FIP File (VALMSG)</t>
+          <t>X-Checks Publication File</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>20260602 VALMSG (Accounting Principle).xlsx</t>
+          <t>20260313 Cross Checks All.xlsx</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>FIP Methods Rules and Condition</t>
+          <t>cross checks all</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1586,22 +1685,22 @@
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Conditions</t>
+          <t>Grouping By</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>X-Checks Publication File</t>
+          <t>Mapping File</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>20260313 Cross Checks All - Copy.xlsx</t>
+          <t>Mapping Table with 20 rows.txt</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>cross checks all</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1613,22 +1712,22 @@
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Conditions</t>
+          <t>Accounting Principles</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>FIP File</t>
+          <t>Validation Methods File</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>20260602 VALMETH (Conditions).xlsx</t>
+          <t>validation methods.xlsx</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>FIP Conditions</t>
+          <t>Validation Methods</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -1640,22 +1739,22 @@
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Accounting Principles</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>FIP File (ZQ9_VALFLDGR)</t>
+          <t>X-Checks Publication File</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>VALFLDGR file with 12348 Data rows on sheet Sheet1.XLSX</t>
+          <t>20260602 VALMSG (Accounting Principle).xlsx</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Sheet1</t>
+          <t>cross checks all</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1667,22 +1766,22 @@
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Accounting Principles</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>X-Checks Publication File</t>
+          <t>FIP File (VALMSG)</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>20260313 Cross Checks All.xlsx</t>
+          <t>20260602 VALMSG (Accounting Principle).xlsx</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>cross checks all</t>
+          <t>FIP Methods Rules and Condition</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -1694,22 +1793,22 @@
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Conditions</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Mapping File</t>
+          <t>X-Checks Publication File</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Mapping Table with 20 rows.txt</t>
+          <t>20260313 Cross Checks All - Copy.xlsx</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>cross checks all</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1721,22 +1820,22 @@
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Conditions</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Validation Methods File</t>
+          <t>FIP File</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>validation methods.xlsx</t>
+          <t>20260602 VALMETH (Conditions).xlsx</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Validation Methods</t>
+          <t>FIP Conditions</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -1753,17 +1852,17 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>FIP File (VALMSG)</t>
+          <t>FIP file</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>20260602 VALMSG (Accounting Principle).xlsx</t>
+          <t>20260318 FIP X-Checks.txt</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>FIP Methods Rules and Condition</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1780,178 +1879,213 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
+          <t>FIP File (ZQ9_VALFLDGR)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>VALFLDGR file with 12348 Data rows on sheet Sheet1.XLSX</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Sheet1</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>X-Checks Publication File</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>20260313 Cross Checks All.xlsx</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>cross checks all</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Mapping File</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Mapping Table with 20 rows.txt</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Validation Methods File</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>validation methods.xlsx</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Validation Methods</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>FIP File (VALMSG)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>20260602 VALMSG (Accounting Principle).xlsx</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>FIP Methods Rules and Condition</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
           <t>FIP File</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>20260602 VALMETH (Conditions).xlsx</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>FIP Conditions</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="25.5" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="23" ht="25.5" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>General UI and Dialog Behavior Test Cases</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Tested Date</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="51" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Splash screen on launch</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Double-click X-Checks_v1.0.0.exe.</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Splash screen displays with version v1.0.0 and closes automatically when the main window is ready.</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr"/>
-      <c r="E20" s="7" t="inlineStr"/>
-      <c r="F20" s="7" t="inlineStr"/>
-    </row>
-    <row r="21" ht="51" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Task selector title</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Observe the task selector window title and heading label.</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Title bar and heading both read 'X-Check Application v1.0.0'.</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr"/>
-      <c r="E21" s="7" t="inlineStr"/>
-      <c r="F21" s="7" t="inlineStr"/>
-    </row>
-    <row r="22" ht="51" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Dropdown population</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Open the task selector dropdown.</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Four options present: Grouping By, Accounting Principles, Conditions, Full Run — in that order.</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr"/>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="7" t="inlineStr"/>
-    </row>
-    <row r="23" ht="51" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>Start button disabled by default</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Open the app without selecting a task.</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Start button is disabled (greyed out).</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr"/>
-      <c r="E23" s="7" t="inlineStr"/>
-      <c r="F23" s="7" t="inlineStr"/>
-    </row>
-    <row r="24" ht="51" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Start button enables on selection</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Select any task from the dropdown.</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Start button becomes enabled immediately.</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr"/>
-      <c r="E24" s="7" t="inlineStr"/>
-      <c r="F24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="51" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Close task selector</t>
+          <t>Splash screen on launch</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Click the red X on the task selector.</t>
+          <t>Double-click X-Checks_v1.0.0.exe.</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Application exits cleanly — no error dialogs, no orphaned processes.</t>
+          <t>Splash screen displays with version v1.0.0 and closes automatically when the main window is ready.</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr"/>
@@ -1961,17 +2095,17 @@
     <row r="26" ht="51" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Upload dialog title</t>
+          <t>Task selector title</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Select each strategy in turn and click Start.</t>
+          <t>Observe the task selector window title and heading label.</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Upload dialog title matches the strategy: 'Grouping By Files', 'Accounting Principles Files', 'Conditions Files', 'Full Run — All Strategies'.</t>
+          <t>Title bar and heading both read 'X-Check Application v1.0.0'.</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr"/>
@@ -1981,17 +2115,17 @@
     <row r="27" ht="51" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Advisory sheet-name label</t>
+          <t>Dropdown population</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Open any upload dialog that has sheet name fields.</t>
+          <t>Open the task selector dropdown.</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Centred black label reads 'If the sheet name changes from the current default in the Excel workbook, update it manually.'</t>
+          <t>Five options present: X-Checks, Grouping By, Accounting Principles, Conditions, Full Run — in that order.</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr"/>
@@ -2001,17 +2135,17 @@
     <row r="28" ht="51" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Proceed disabled until all files provided</t>
+          <t>Start button disabled by default</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Open upload dialog; fill in only some required fields.</t>
+          <t>Open the app without selecting a task.</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Proceed button stays disabled until all required fields and output directory are provided.</t>
+          <t>Start button is disabled (greyed out).</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr"/>
@@ -2021,17 +2155,17 @@
     <row r="29" ht="51" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Cancel upload dialog returns to selector</t>
+          <t>Start button enables on selection</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Open upload dialog and close it with the red X.</t>
+          <t>Select any task from the dropdown.</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Task selector reappears; Start button returns to disabled state.</t>
+          <t>Start button becomes enabled immediately.</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr"/>
@@ -2041,17 +2175,17 @@
     <row r="30" ht="51" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Progress dialog opens on Proceed</t>
+          <t>Close task selector</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Complete all required fields and click Proceed.</t>
+          <t>Click the red X on the task selector.</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Progress dialog opens with scrollable log; Stop button visible.</t>
+          <t>Application exits cleanly — no error dialogs, no orphaned processes.</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr"/>
@@ -2061,17 +2195,17 @@
     <row r="31" ht="51" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Progress dialog — error style</t>
+          <t>Upload dialog title</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Trigger a file-not-found error (rename a file after selecting it).</t>
+          <t>Select each strategy in turn and click Start.</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Error line appears in bold red text; Windows error chime plays; Exit Application button appears.</t>
+          <t>Upload dialog title matches the strategy: 'X-Check Files', 'Grouping By Files', 'Accounting Principles Files', 'Conditions Files', 'Full Run — All Strategies'.</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr"/>
@@ -2081,17 +2215,17 @@
     <row r="32" ht="51" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Return to Form after error</t>
+          <t>Advisory sheet-name label</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>After an error, click 'Return to Form'.</t>
+          <t>Open any upload dialog that has sheet name fields.</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Upload dialog re-opens with all previously entered paths pre-filled.</t>
+          <t>Centred black label reads 'If the sheet name changes from the current default in the Excel workbook, update it manually.'</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr"/>
@@ -2101,76 +2235,97 @@
     <row r="33" ht="51" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Stop button halts processing</t>
+          <t>Proceed disabled until all files provided</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Start a run and click Stop.</t>
+          <t>Open upload dialog; fill in only some required fields.</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Processing halts cleanly; log shows 'Processing halted by user.'; Return to Form button appears.</t>
+          <t>Proceed button stays disabled until all required fields and output directory are provided.</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr"/>
       <c r="E33" s="7" t="inlineStr"/>
       <c r="F33" s="7" t="inlineStr"/>
     </row>
-    <row r="35" ht="25.5" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Detailed Field Interaction Test Cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>Tested By</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>Tested Date</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
+    <row r="34" ht="51" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Cancel upload dialog returns to selector</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Open upload dialog and close it with the red X.</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Task selector reappears; Start button returns to disabled state.</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr"/>
+      <c r="E34" s="7" t="inlineStr"/>
+      <c r="F34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35" ht="51" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Progress dialog opens on Proceed</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Complete all required fields and click Proceed.</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Progress dialog opens with scrollable log; Stop button visible.</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr"/>
+      <c r="E35" s="7" t="inlineStr"/>
+      <c r="F35" s="7" t="inlineStr"/>
+    </row>
+    <row r="36" ht="51" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Progress dialog — error style</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Trigger a file-not-found error (rename a file after selecting it).</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Error line appears in bold red text; Windows error chime plays; Exit Application button appears.</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr"/>
+      <c r="E36" s="7" t="inlineStr"/>
+      <c r="F36" s="7" t="inlineStr"/>
     </row>
     <row r="37" ht="51" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Required field asterisk label</t>
+          <t>Return to Form after error</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Open any upload dialog.</t>
+          <t>After an error, click 'Return to Form'.</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Required fields show label text ending in ' *'; output directory shows 'Output Directory *'.</t>
+          <t>Upload dialog re-opens with all previously entered paths pre-filled.</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr"/>
@@ -2180,97 +2335,76 @@
     <row r="38" ht="51" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Browse button opens file picker</t>
+          <t>Stop button halts processing</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Click Browse next to any file field.</t>
+          <t>Start a run and click Stop.</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>OS file picker dialog opens filtered to the correct file type (e.g. Excel Files *.xlsx).</t>
+          <t>Processing halts cleanly; log shows 'Processing halted by user.'; Return to Form button appears.</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr"/>
       <c r="E38" s="7" t="inlineStr"/>
       <c r="F38" s="7" t="inlineStr"/>
     </row>
-    <row r="39" ht="51" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>File selected — path label updates</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Select a file via Browse.</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Path label updates to the filename (not the full path); text turns black.</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr"/>
-      <c r="E39" s="7" t="inlineStr"/>
-      <c r="F39" s="7" t="inlineStr"/>
-    </row>
-    <row r="40" ht="51" customHeight="1">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>Sheet name field enables on file select</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>Select a file for a field that has a sheet name input.</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>Sheet name entry becomes editable; text turns black.</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="inlineStr"/>
-      <c r="E40" s="7" t="inlineStr"/>
-      <c r="F40" s="7" t="inlineStr"/>
-    </row>
-    <row r="41" ht="51" customHeight="1">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>Sheet name retains default until edited</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Select a file without changing the sheet name.</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>Sheet name field shows the configured default (e.g. 'cross checks all', 'Sheet1').</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr"/>
-      <c r="E41" s="7" t="inlineStr"/>
-      <c r="F41" s="7" t="inlineStr"/>
+    <row r="40" ht="25.5" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Detailed Field Interaction Test Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Tested By</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Tested Date</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="51" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>Output directory Browse</t>
+          <t>Required field asterisk label</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Click Browse next to Output Directory.</t>
+          <t>Open any upload dialog.</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Folder picker opens; selected path shows in full in the label.</t>
+          <t>Required fields show label text ending in ' *'; output directory shows 'Output Directory *'.</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr"/>
@@ -2280,17 +2414,17 @@
     <row r="43" ht="51" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>Process only differences — default ON</t>
+          <t>Browse button opens file picker</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Open any upload dialog.</t>
+          <t>Click Browse next to any file field.</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>'Process only differences' checkbox is ticked by default.</t>
+          <t>OS file picker dialog opens filtered to the correct file type (e.g. Excel Files *.xlsx).</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr"/>
@@ -2300,196 +2434,171 @@
     <row r="44" ht="51" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>Dialog position</t>
+          <t>File selected — path label updates</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Move the task selector to a corner of the screen, then open the upload dialog.</t>
+          <t>Select a file via Browse.</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Upload dialog appears at the same position as the task selector, clamped within the usable screen area.</t>
+          <t>Path label updates to the filename (not the full path); text turns black.</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr"/>
       <c r="E44" s="7" t="inlineStr"/>
       <c r="F44" s="7" t="inlineStr"/>
     </row>
-    <row r="46" ht="25.5" customHeight="1">
-      <c r="A46" s="5" t="inlineStr">
-        <is>
-          <t>Workflow-Specific Test Cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
-        <is>
-          <t>Workflow</t>
-        </is>
-      </c>
-      <c r="B47" s="6" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>Tested By</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>Tested Date</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
+    <row r="45" ht="51" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Sheet name field enables on file select</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Select a file for a field that has a sheet name input.</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Sheet name entry becomes editable; text turns black.</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr"/>
+      <c r="E45" s="7" t="inlineStr"/>
+      <c r="F45" s="7" t="inlineStr"/>
+    </row>
+    <row r="46" ht="51" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Sheet name retains default until edited</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Select a file without changing the sheet name.</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Sheet name field shows the configured default (e.g. 'cross checks all', 'Sheet1').</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr"/>
+      <c r="E46" s="7" t="inlineStr"/>
+      <c r="F46" s="7" t="inlineStr"/>
+    </row>
+    <row r="47" ht="51" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Output directory Browse</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Click Browse next to Output Directory.</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Folder picker opens; selected path shows in full in the label.</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr"/>
+      <c r="E47" s="7" t="inlineStr"/>
+      <c r="F47" s="7" t="inlineStr"/>
     </row>
     <row r="48" ht="51" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>Grouping By</t>
+          <t>Process only differences — default ON</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>End-to-end run completes</t>
+          <t>Open any upload dialog.</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Run debug EXE with test data.</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>Output workbook produced in ~/Downloads/Output; 7 sheets present; no error lines in log.</t>
-        </is>
-      </c>
+          <t>'Process only differences' checkbox is ticked by default.</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr"/>
       <c r="E48" s="7" t="inlineStr"/>
       <c r="F48" s="7" t="inlineStr"/>
-      <c r="G48" s="7" t="inlineStr"/>
     </row>
     <row r="49" ht="51" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>Grouping By</t>
+          <t>Dialog position</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Compare sheet contains results</t>
+          <t>Move the task selector to a corner of the screen, then open the upload dialog.</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Open output workbook → Compare sheet.</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>Result column contains 'Matched' and/or 'Not in FIP' values; row count &gt; 0.</t>
-        </is>
-      </c>
+          <t>Upload dialog appears at the same position as the task selector, clamped within the usable screen area.</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr"/>
       <c r="E49" s="7" t="inlineStr"/>
       <c r="F49" s="7" t="inlineStr"/>
-      <c r="G49" s="7" t="inlineStr"/>
-    </row>
-    <row r="50" ht="51" customHeight="1">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>Grouping By</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>FIP - Processed has Key column</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>Open FIP - Processed sheet.</t>
-        </is>
-      </c>
-      <c r="D50" s="7" t="inlineStr">
-        <is>
-          <t>Column 'Key' present; values follow 'ValidRule|EBX Item' format.</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr"/>
-      <c r="F50" s="7" t="inlineStr"/>
-      <c r="G50" s="7" t="inlineStr"/>
-    </row>
-    <row r="51" ht="51" customHeight="1">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>Grouping By</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>EBX - Processed stacks Grouping By values</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>Open EBX - Processed sheet.</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>Each Grouping By value appears as a separate row with a Key column.</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr"/>
-      <c r="F51" s="7" t="inlineStr"/>
-      <c r="G51" s="7" t="inlineStr"/>
-    </row>
-    <row r="52" ht="51" customHeight="1">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>Grouping By</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>Mapping File sheet matches input</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>Open Mapping File sheet.</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>Two columns: FIP Data and EBX item; row count matches input mapping file.</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr"/>
-      <c r="F52" s="7" t="inlineStr"/>
-      <c r="G52" s="7" t="inlineStr"/>
+    </row>
+    <row r="51" ht="25.5" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Workflow-Specific Test Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>Tested By</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>Tested Date</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="51" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Accounting Principles</t>
+          <t>X-Checks</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -2504,7 +2613,7 @@
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Output workbook produced in ~/Downloads/Output; 4 sheets present; no error lines in log.</t>
+          <t>Output workbook produced in ~/Downloads/Output; 2 sheets present; no error lines in log.</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr"/>
@@ -2514,22 +2623,22 @@
     <row r="54" ht="51" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>Accounting Principles</t>
+          <t>X-Checks</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Comparison sheet formatting</t>
+          <t>X-Checks Comparison sheet present</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Open Comparison sheet.</t>
+          <t>Open output workbook.</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Match rows have green fill + green text; MisMatch rows have red fill + red text.</t>
+          <t>Sheet named 'X-Checks Comparison' present with rows of comparison data.</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr"/>
@@ -2539,22 +2648,22 @@
     <row r="55" ht="51" customHeight="1">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>Accounting Principles</t>
+          <t>X-Checks</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Method bindings extracted</t>
+          <t>Result column colour-coded</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Check progress log.</t>
+          <t>Open X-Checks Comparison sheet.</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Log line 'Validation Methods — Method bindings extracted N' with N &gt; 0.</t>
+          <t>Result column contains formatted values (Matched / MisMatch / Not Found); conditional formatting applied.</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr"/>
@@ -2564,22 +2673,22 @@
     <row r="56" ht="51" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>Accounting Principles</t>
+          <t>X-Checks</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>In-scope X-Checks logged</t>
+          <t>Optional files handled gracefully</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Check progress log.</t>
+          <t>Run with only required files (no GCoA or Known Exception List).</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Log line 'EBX — In-scope X-Check Nos N' with N &gt; 0.</t>
+          <t>Run completes without error; log notes optional files were skipped.</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr"/>
@@ -2589,22 +2698,22 @@
     <row r="57" ht="51" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>Conditions</t>
+          <t>X-Checks</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>End-to-end run completes</t>
+          <t>Experimental checkboxes visible</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Run debug EXE with test data.</t>
+          <t>Open X-Checks upload dialog.</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Output workbook produced in ~/Downloads/Output; 4 sheets present; no error lines in log.</t>
+          <t>Two experimental checkboxes present: 'Apply Version Spanning Validation' and 'Apply Prior Year Balance Formula', both unchecked by default.</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr"/>
@@ -2614,22 +2723,22 @@
     <row r="58" ht="51" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>Conditions</t>
+          <t>Grouping By</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>Summary block present</t>
+          <t>End-to-end run completes</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Open Conditions sheet.</t>
+          <t>Run debug EXE with test data.</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Top rows show summary: Total Pairs, Matched (TRUE), Not Matched (FALSE) before data rows.</t>
+          <t>Output workbook produced in ~/Downloads/Output; 7 sheets present; no error lines in log.</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr"/>
@@ -2639,22 +2748,22 @@
     <row r="59" ht="51" customHeight="1">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>Conditions</t>
+          <t>Grouping By</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Conditions sheet has TRUE and FALSE rows</t>
+          <t>Compare sheet contains results</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Inspect Comparison column in Conditions sheet.</t>
+          <t>Open output workbook → Compare sheet.</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Column contains TRUE and/or FALSE values; EBX Data column contains XCheck|Condition format keys.</t>
+          <t>Result column contains 'Matched' and/or 'Not in FIP' values; row count &gt; 0.</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr"/>
@@ -2664,22 +2773,22 @@
     <row r="60" ht="51" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>Conditions</t>
+          <t>Grouping By</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>Working Sheet has concat columns</t>
+          <t>FIP - Processed has Key column</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Open Working Sheet.</t>
+          <t>Open FIP - Processed sheet.</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Columns present for each of the 5 condition types plus corresponding '(Concat)' columns.</t>
+          <t>Column 'Key' present; values follow 'ValidRule|EBX Item' format.</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr"/>
@@ -2689,22 +2798,22 @@
     <row r="61" ht="51" customHeight="1">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Grouping By</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>End-to-end run completes</t>
+          <t>EBX - Processed stacks Grouping By values</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Run debug EXE with test data.</t>
+          <t>Open EBX - Processed sheet.</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Single combined output workbook produced in ~/Downloads/Output; 13 sheets present; no error lines in log.</t>
+          <t>Each Grouping By value appears as a separate row with a Key column.</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr"/>
@@ -2714,22 +2823,22 @@
     <row r="62" ht="51" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Grouping By</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>All three strategies execute in order</t>
+          <t>Mapping File sheet matches input</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Check progress log.</t>
+          <t>Open Mapping File sheet.</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Log shows '— Starting: Grouping By —', then '— Starting: Accounting Principles —', then '— Starting: Conditions —' in sequence.</t>
+          <t>Two columns: FIP Data and EBX item; row count matches input mapping file.</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr"/>
@@ -2739,22 +2848,22 @@
     <row r="63" ht="51" customHeight="1">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Accounting Principles</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Sheet tab colours</t>
+          <t>End-to-end run completes</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Open combined workbook and inspect tab colours.</t>
+          <t>Run debug EXE with test data.</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>GB tabs = orange; AP tabs = dark blue; Cond tabs = Zurich blue; Processing Log = grey.</t>
+          <t>Output workbook produced in ~/Downloads/Output; 4 sheets present; no error lines in log.</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr"/>
@@ -2764,22 +2873,22 @@
     <row r="64" ht="51" customHeight="1">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Accounting Principles</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>Tab prefixes</t>
+          <t>Comparison sheet formatting</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>Inspect sheet tab names.</t>
+          <t>Open Comparison sheet.</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Grouping By sheets prefixed 'GB — '; Accounting Principles prefixed 'AP — '; Conditions prefixed 'Cond — '.</t>
+          <t>Match rows have green fill + green text; MisMatch rows have red fill + red text.</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr"/>
@@ -2789,22 +2898,22 @@
     <row r="65" ht="51" customHeight="1">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Accounting Principles</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Combined workbook sheet count</t>
+          <t>Method bindings extracted</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Count sheets in combined workbook.</t>
+          <t>Check progress log.</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>13 sheets: 6 (GB) + 3 (AP) + 3 (Cond) + 1 (Processing Log).</t>
+          <t>Log line 'Validation Methods — Method bindings extracted N' with N &gt; 0.</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr"/>
@@ -2814,22 +2923,22 @@
     <row r="66" ht="51" customHeight="1">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>Full Run</t>
+          <t>Accounting Principles</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>Processing Log spans all strategies</t>
+          <t>In-scope X-Checks logged</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>Open Processing Log sheet.</t>
+          <t>Check progress log.</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Log contains entries from all three strategies in sequence — no gaps or missing strategy sections.</t>
+          <t>Log line 'EBX — In-scope X-Check Nos N' with N &gt; 0.</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr"/>
@@ -2839,22 +2948,22 @@
     <row r="67" ht="51" customHeight="1">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>All strategies</t>
+          <t>Conditions</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Sensitivity label applied</t>
+          <t>End-to-end run completes</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Open any output workbook in Excel, check File → Info → Protect Workbook.</t>
+          <t>Run debug EXE with test data.</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Microsoft Information Protection label 'Internal Use Only' is applied to the workbook.</t>
+          <t>Output workbook produced in ~/Downloads/Output; 4 sheets present; no error lines in log.</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr"/>
@@ -2864,27 +2973,277 @@
     <row r="68" ht="51" customHeight="1">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>All strategies</t>
+          <t>Conditions</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>Version stamp in log</t>
+          <t>Summary block present</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>Open Processing Log sheet of any output workbook.</t>
+          <t>Open Conditions sheet.</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>First row of log reads 'System — X-Check Application v1.0.0'.</t>
+          <t>Top rows show summary: Total Pairs, Matched (TRUE), Not Matched (FALSE) before data rows.</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr"/>
       <c r="F68" s="7" t="inlineStr"/>
       <c r="G68" s="7" t="inlineStr"/>
+    </row>
+    <row r="69" ht="51" customHeight="1">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>Conditions</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Conditions sheet has TRUE and FALSE rows</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Inspect Comparison column in Conditions sheet.</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Column contains TRUE and/or FALSE values; EBX Data column contains XCheck|Condition format keys.</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr"/>
+      <c r="F69" s="7" t="inlineStr"/>
+      <c r="G69" s="7" t="inlineStr"/>
+    </row>
+    <row r="70" ht="51" customHeight="1">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>Conditions</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Working Sheet has concat columns</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Open Working Sheet.</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>Columns present for each of the 5 condition types plus corresponding '(Concat)' columns.</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr"/>
+      <c r="F70" s="7" t="inlineStr"/>
+      <c r="G70" s="7" t="inlineStr"/>
+    </row>
+    <row r="71" ht="51" customHeight="1">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>End-to-end run completes</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Run debug EXE with test data.</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>Single combined output workbook produced in ~/Downloads/Output; 13 sheets present; no error lines in log.</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr"/>
+      <c r="F71" s="7" t="inlineStr"/>
+      <c r="G71" s="7" t="inlineStr"/>
+    </row>
+    <row r="72" ht="51" customHeight="1">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>All four strategies execute in order</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Check progress log.</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Log shows '— Starting: X-Checks —', then '— Starting: Grouping By —', then '— Starting: Accounting Principles —', then '— Starting: Conditions —' in sequence.</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr"/>
+      <c r="F72" s="7" t="inlineStr"/>
+      <c r="G72" s="7" t="inlineStr"/>
+    </row>
+    <row r="73" ht="51" customHeight="1">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Sheet tab colours</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Open combined workbook and inspect tab colours.</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>XC tabs = green; GB tabs = orange; AP tabs = dark blue; Cond tabs = Zurich blue; Processing Log = grey.</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr"/>
+      <c r="F73" s="7" t="inlineStr"/>
+      <c r="G73" s="7" t="inlineStr"/>
+    </row>
+    <row r="74" ht="51" customHeight="1">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Tab prefixes</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>Inspect sheet tab names.</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>X-Checks prefixed 'XC — '; Grouping By prefixed 'GB — '; Accounting Principles prefixed 'AP — '; Conditions prefixed 'Cond — '.</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr"/>
+      <c r="F74" s="7" t="inlineStr"/>
+      <c r="G74" s="7" t="inlineStr"/>
+    </row>
+    <row r="75" ht="51" customHeight="1">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Combined workbook sheet count</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Count sheets in combined workbook.</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>15 sheets: 1 (XC) + 6 (GB) + 3 (AP) + 3 (Cond) + 1 (Processing Log) = 14 data sheets + 1 log.</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr"/>
+      <c r="F75" s="7" t="inlineStr"/>
+      <c r="G75" s="7" t="inlineStr"/>
+    </row>
+    <row r="76" ht="51" customHeight="1">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>Full Run</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Processing Log spans all strategies</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Open Processing Log sheet.</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>Log contains entries from all four strategies in sequence — no gaps or missing strategy sections.</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr"/>
+      <c r="F76" s="7" t="inlineStr"/>
+      <c r="G76" s="7" t="inlineStr"/>
+    </row>
+    <row r="77" ht="51" customHeight="1">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>All strategies</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Sensitivity label applied</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Open any output workbook in Excel, check File → Info → Protect Workbook.</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Information Protection label 'Internal Use Only' is applied to the workbook.</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr"/>
+      <c r="F77" s="7" t="inlineStr"/>
+      <c r="G77" s="7" t="inlineStr"/>
+    </row>
+    <row r="78" ht="51" customHeight="1">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>All strategies</t>
+        </is>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Version stamp in log</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Open Processing Log sheet of any output workbook.</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>First row of log reads 'System — X-Check Application v1.0.0'.</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr"/>
+      <c r="F78" s="7" t="inlineStr"/>
+      <c r="G78" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>